<commit_message>
Update Dashboard KPIs, Reception form units to Tons, add Merma tracking, and add management features
</commit_message>
<xml_diff>
--- a/data/base_datos.xlsx
+++ b/data/base_datos.xlsx
@@ -563,16 +563,6 @@
           <t>C01</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>Aleta 500-1000</t>
@@ -1046,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1060,88 +1050,244 @@
           <t>Nombre_Lider</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Num_Operarios</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cuadrilla 1</t>
-        </is>
-      </c>
+          <t>Cuadrilla 2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cuadrilla 2</t>
-        </is>
-      </c>
+          <t>Cuadrilla 3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cuadrilla 3</t>
-        </is>
-      </c>
+          <t>Cuadrilla 4</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cuadrilla 4</t>
-        </is>
-      </c>
+          <t>Cuadrilla 5</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cuadrilla 5</t>
-        </is>
-      </c>
+          <t>Cuadrilla 6</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cuadrilla 6</t>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Envasado</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cuadrilla 7</t>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Envasado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>rodriguez</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Envasado</t>
         </is>
       </c>
     </row>

</xml_diff>